<commit_message>
Daily EOD data and reports for 2026-08-26
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260826.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260826.xlsx
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.36</v>
+        <v>2.355</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.04</v>
+        <v>-0.045</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.67%</t>
+          <t>-1.87%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>165200</v>
+        <v>164850</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-2800</v>
+        <v>-3150</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>68.48</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.20%</t>
+          <t>1.17%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>757731.2</v>
+        <v>757509.9</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>8962.65</v>
+        <v>8741.35</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>157.76</v>
+        <v>157.84</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.75</v>
+        <v>0.83</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.48%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1.05</v>
+        <v>1.045</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>0.97%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>10500</v>
+        <v>10450</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>174.39</v>
+        <v>174.45</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.75</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>0.47%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>697560</v>
+        <v>697800</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3000</v>
+        <v>3240</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0</v>
+        <v>0.285</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.285</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0</v>
+        <v>5700</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-5700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.29</v>
+        <v>34.32</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.79%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.63</v>
+        <v>31.57</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-1.37</v>
+        <v>-1.43</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-4.15%</t>
+          <t>-4.33%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>40739.44</v>
+        <v>40662.16</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-1764.56</v>
+        <v>-1841.84</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1975025.39</v>
+        <v>1980266.8</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-53996.8</v>
+        <v>-48755.38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>